<commit_message>
se suben todos los archivos, no solo el md
</commit_message>
<xml_diff>
--- a/aym_productos/Inventario.xlsx
+++ b/aym_productos/Inventario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sergio\Desktop\AyMTodoEscolarWEBSITE\aym_productos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{805E29C0-B489-41E4-94AC-61193581A77B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB4AC7DA-0379-4BD2-A3C1-44D6CFCEC17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19320" yWindow="-2100" windowWidth="19440" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inventario" sheetId="3" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1828" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1829" uniqueCount="570">
   <si>
     <t>PRODUCTO</t>
   </si>
@@ -5084,60 +5084,6 @@
   </cellStyles>
   <dxfs count="13">
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" readingOrder="0"/>
-      <border outline="0">
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="\$\ #,##0"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79998168889431442"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC000"/>
@@ -5251,6 +5197,60 @@
         <top/>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" readingOrder="0"/>
+      <border outline="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="\$\ #,##0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -5522,29 +5522,29 @@
   <autoFilter ref="A1:E604" xr:uid="{798956E9-E668-49C2-AF4D-5ADB45684FAD}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{0BE28364-A577-4E9E-B6BC-99DD0C310438}" name="PRODUCTO"/>
-    <tableColumn id="2" xr3:uid="{AE5BA1E0-66FC-48D8-9459-B939FBD9F7BB}" name="CANTIDAD" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{AD921975-2956-4F70-98F8-FFD4FA3BD50D}" name="COSTO" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{D46F3205-8F5D-4219-8634-56AC91255DBD}" name="COSTO TOTAL" dataDxfId="1">
+    <tableColumn id="2" xr3:uid="{AE5BA1E0-66FC-48D8-9459-B939FBD9F7BB}" name="CANTIDAD" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{AD921975-2956-4F70-98F8-FFD4FA3BD50D}" name="COSTO" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{D46F3205-8F5D-4219-8634-56AC91255DBD}" name="COSTO TOTAL" dataDxfId="7">
       <calculatedColumnFormula>Tabla4[[#This Row],[CANTIDAD]]*Tabla4[[#This Row],[COSTO]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{A4651438-3CC9-4FE4-A9DF-CFDBB0E7A241}" name="P.VENTA" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{A4651438-3CC9-4FE4-A9DF-CFDBB0E7A241}" name="P.VENTA" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FFE6C29C-19F5-4E6F-9FD2-F082E539CBCC}" name="Tabla1" displayName="Tabla1" ref="A1:E222" totalsRowShown="0" headerRowDxfId="9" tableBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FFE6C29C-19F5-4E6F-9FD2-F082E539CBCC}" name="Tabla1" displayName="Tabla1" ref="A1:E222" totalsRowShown="0" headerRowDxfId="5" tableBorderDxfId="4">
   <autoFilter ref="A1:E222" xr:uid="{FFE6C29C-19F5-4E6F-9FD2-F082E539CBCC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E222">
     <sortCondition ref="B1:B222"/>
   </sortState>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{9E9AF278-7242-4C43-B19D-5626AB3E7448}" name="Código"/>
-    <tableColumn id="2" xr3:uid="{2CF3BA67-51DF-4F76-971A-AB56CB7A8846}" name="Producto" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{8FF6691C-DA54-4A87-95D8-408A286B3455}" name="Cantidad" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{A4CA90C9-2854-4AE5-9D91-A78A42901785}" name="Precio Unitario" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{762C3A23-E954-450E-98E9-AB0055F64C17}" name="Precio Total" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{2CF3BA67-51DF-4F76-971A-AB56CB7A8846}" name="Producto" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{8FF6691C-DA54-4A87-95D8-408A286B3455}" name="Cantidad" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{A4CA90C9-2854-4AE5-9D91-A78A42901785}" name="Precio Unitario" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{762C3A23-E954-450E-98E9-AB0055F64C17}" name="Precio Total" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5816,7 +5816,7 @@
   <sheetPr>
     <tabColor rgb="FF00B050"/>
   </sheetPr>
-  <dimension ref="A1:F604"/>
+  <dimension ref="A1:F605"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46.5703125" customWidth="1"/>
@@ -12443,7 +12443,9 @@
       <c r="A316" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="B316" s="61"/>
+      <c r="B316" s="61">
+        <v>1</v>
+      </c>
       <c r="C316" s="6"/>
       <c r="D316" s="68">
         <f>Tabla4[[#This Row],[CANTIDAD]]*Tabla4[[#This Row],[COSTO]]</f>
@@ -18056,8 +18058,11 @@
         <v>3180</v>
       </c>
       <c r="E604" s="51"/>
-      <c r="F604" s="108"/>
-    </row>
+      <c r="F604" s="108" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="605" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="F1:F603" xr:uid="{0711EC33-1702-4843-AFFD-90F6BFF60306}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>